<commit_message>
Patička na podlaze pod stránkami, bez čísel stránek, větší a jasnější záložky
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011AtHpjbqs9iMR23airjHG2
</commit_message>
<xml_diff>
--- a/examples/fyzioterapie/ladne-web.xlsx
+++ b/examples/fyzioterapie/ladne-web.xlsx
@@ -8122,26 +8122,8 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>show_folio</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="C19" s="13" t="inlineStr">
-        <is>
-          <t>yes / no</t>
-        </is>
-      </c>
-      <c r="D19" s="13" t="inlineStr">
-        <is>
-          <t>Zobrazit malé číslo stránky (02 / 05) nahoře.</t>
-        </is>
-      </c>
+      <c r="C19" s="15" t="n"/>
+      <c r="D19" s="15" t="n"/>
     </row>
     <row r="20">
       <c r="C20" s="15" t="n"/>

</xml_diff>

<commit_message>
Barevné profily: doplňkové pozadí, šedá, Tron
</commit_message>
<xml_diff>
--- a/examples/fyzioterapie/ladne-web.xlsx
+++ b/examples/fyzioterapie/ladne-web.xlsx
@@ -1437,7 +1437,7 @@
       <c r="B60" s="5" t="inlineStr"/>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech. Teplá cihlová.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Teplá cihlová.</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
@@ -1455,7 +1455,7 @@
       <c r="B61" s="5" t="inlineStr"/>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech. Medová, zlatavá.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Medová, zlatavá.</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
@@ -1473,7 +1473,7 @@
       <c r="B62" s="5" t="inlineStr"/>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech. Svěží korálová.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Svěží korálová.</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
@@ -1491,7 +1491,7 @@
       <c r="B63" s="5" t="inlineStr"/>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech. Jemná broskvová.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Jemná broskvová.</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
@@ -1509,7 +1509,7 @@
       <c r="B64" s="5" t="inlineStr"/>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech. Karamelově hnědá.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Karamelově hnědá.</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
@@ -1527,7 +1527,7 @@
       <c r="B65" s="5" t="inlineStr"/>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech. Prášková růže.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Prášková růže.</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
@@ -1545,7 +1545,7 @@
       <c r="B66" s="5" t="inlineStr"/>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech. Hluboká vínová.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Hluboká vínová.</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
@@ -1563,7 +1563,7 @@
       <c r="B67" s="5" t="inlineStr"/>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech. Světlý písek.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Světlý písek.</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
@@ -1575,36 +1575,36 @@
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>tron</t>
+          <t>seda</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr"/>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>Neonově azurová s oranžovou, ubíhající mřížka v pozadí.</t>
+          <t>Stupně šedi, bez barvy. Pozadí v tmavě šedých tónech.</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>#00E5FF · #FF7A1A</t>
+          <t>#9C9C9E</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>matrix</t>
+          <t>tron</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr"/>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Fosforově zelená, jemně padající znaky v pozadí.</t>
+          <t>Neonově azurová s oranžovou, záře na hranách, pozadí v modrých a oranžových tónech.</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>#00FF41</t>
+          <t>#00E5FF · #FF7A1A</t>
         </is>
       </c>
     </row>
@@ -9169,7 +9169,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Neznámý profil" error="Vyberte jeden z nabízených profilů." type="list">
-      <formula1>"manual,terakota,jantar,koral,broskev,karamel,ruze,vinova,pisek,tron,matrix,soumrak,zeme,pastel,sever"</formula1>
+      <formula1>"manual,terakota,jantar,koral,broskev,karamel,ruze,vinova,pisek,seda,tron,soumrak,zeme,pastel,sever"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>